<commit_message>
Count sheet: split Jobs4ECPs and Job-Opportunities by role, like Indeed
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01K4dgNSErFJEdk2fo96NF3d
</commit_message>
<xml_diff>
--- a/docs/market-count-sheet.xlsx
+++ b/docs/market-count-sheet.xlsx
@@ -578,7 +578,7 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Use only what any visitor can see on the public pages, with no sign in and no member access. Type the total number of open ads into Open. If the site lets you sort by date or filter to the last 7 days, type that count into New 7 days. If not, leave it blank. Never use anything from a members only board.</t>
+          <t>Same idea as Indeed, one row per role, using only what any visitor can see on the public pages, with no sign in and no member access. If the site has a search box, type the words in column B. If it only has a role or category filter, use the closest one and write which in the Notes. Type the total number of open ads into Open. If the site lets you sort by date or filter to the last 7 days, type that count into New 7 days. If not, leave it blank. A role with no matching search or filter stays blank. Never use anything from a members only board.</t>
         </is>
       </c>
     </row>
@@ -590,7 +590,7 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Look at the first 20 results of any one Indeed search. Count how many really are eye care roles, and put that as a share (for example 16 of 20 is 0.8) into the Summary sheet, cell B7. Searches pull in some unrelated jobs, so this keeps the estimate honest.</t>
+          <t>Look at the first 20 results of any one Indeed search. Count how many really are eye care roles, and put that as a share (for example 16 of 20 is 0.8) into the Summary sheet, cell B9. Searches pull in some unrelated jobs, so this keeps the estimate honest.</t>
         </is>
       </c>
     </row>
@@ -641,7 +641,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S21"/>
+  <dimension ref="A1:S31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -794,7 +794,7 @@
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>All jobs</t>
+          <t>optometrist</t>
         </is>
       </c>
       <c r="C5" s="7" t="inlineStr">
@@ -822,12 +822,12 @@
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
         <is>
-          <t>Job-Opportunities (OSI)</t>
+          <t>Jobs4ECPs</t>
         </is>
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>All jobs</t>
+          <t>optician</t>
         </is>
       </c>
       <c r="C6" s="7" t="inlineStr">
@@ -855,12 +855,12 @@
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
         <is>
-          <t>Indeed</t>
+          <t>Jobs4ECPs</t>
         </is>
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>optometrist</t>
+          <t>optometric assistant</t>
         </is>
       </c>
       <c r="C7" s="7" t="inlineStr">
@@ -888,12 +888,12 @@
     <row r="8">
       <c r="A8" s="7" t="inlineStr">
         <is>
-          <t>Indeed</t>
+          <t>Jobs4ECPs</t>
         </is>
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>optician</t>
+          <t>optometric technician</t>
         </is>
       </c>
       <c r="C8" s="7" t="inlineStr">
@@ -921,12 +921,12 @@
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
         <is>
-          <t>Indeed</t>
+          <t>Jobs4ECPs</t>
         </is>
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>optometric assistant</t>
+          <t>ophthalmic assistant</t>
         </is>
       </c>
       <c r="C9" s="7" t="inlineStr">
@@ -954,12 +954,12 @@
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
         <is>
-          <t>Indeed</t>
+          <t>Jobs4ECPs</t>
         </is>
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>optometric technician</t>
+          <t>optical manager</t>
         </is>
       </c>
       <c r="C10" s="7" t="inlineStr">
@@ -987,12 +987,12 @@
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
         <is>
-          <t>Indeed</t>
+          <t>Job-Opportunities (OSI)</t>
         </is>
       </c>
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>ophthalmic assistant</t>
+          <t>optometrist</t>
         </is>
       </c>
       <c r="C11" s="7" t="inlineStr">
@@ -1020,12 +1020,12 @@
     <row r="12">
       <c r="A12" s="7" t="inlineStr">
         <is>
-          <t>Indeed</t>
+          <t>Job-Opportunities (OSI)</t>
         </is>
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>optical manager</t>
+          <t>optician</t>
         </is>
       </c>
       <c r="C12" s="7" t="inlineStr">
@@ -1053,12 +1053,12 @@
     <row r="13">
       <c r="A13" s="7" t="inlineStr">
         <is>
-          <t>Indeed</t>
+          <t>Job-Opportunities (OSI)</t>
         </is>
       </c>
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t>eye care clinic</t>
+          <t>optometric assistant</t>
         </is>
       </c>
       <c r="C13" s="7" t="inlineStr">
@@ -1086,10 +1086,14 @@
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
         <is>
-          <t>(your own)</t>
-        </is>
-      </c>
-      <c r="B14" s="9" t="inlineStr"/>
+          <t>Job-Opportunities (OSI)</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>optometric technician</t>
+        </is>
+      </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
           <t>Canada</t>
@@ -1112,89 +1116,415 @@
       <c r="R14" s="8" t="n"/>
       <c r="S14" s="8" t="n"/>
     </row>
+    <row r="15">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>Job-Opportunities (OSI)</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>ophthalmic assistant</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="n"/>
+      <c r="E15" s="8" t="n"/>
+      <c r="F15" s="8" t="n"/>
+      <c r="G15" s="8" t="n"/>
+      <c r="H15" s="8" t="n"/>
+      <c r="I15" s="8" t="n"/>
+      <c r="J15" s="8" t="n"/>
+      <c r="K15" s="8" t="n"/>
+      <c r="L15" s="8" t="n"/>
+      <c r="M15" s="8" t="n"/>
+      <c r="N15" s="8" t="n"/>
+      <c r="O15" s="8" t="n"/>
+      <c r="P15" s="8" t="n"/>
+      <c r="Q15" s="8" t="n"/>
+      <c r="R15" s="8" t="n"/>
+      <c r="S15" s="8" t="n"/>
+    </row>
     <row r="16">
-      <c r="A16" s="10" t="inlineStr">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>Job-Opportunities (OSI)</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>optical manager</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="D16" s="8" t="n"/>
+      <c r="E16" s="8" t="n"/>
+      <c r="F16" s="8" t="n"/>
+      <c r="G16" s="8" t="n"/>
+      <c r="H16" s="8" t="n"/>
+      <c r="I16" s="8" t="n"/>
+      <c r="J16" s="8" t="n"/>
+      <c r="K16" s="8" t="n"/>
+      <c r="L16" s="8" t="n"/>
+      <c r="M16" s="8" t="n"/>
+      <c r="N16" s="8" t="n"/>
+      <c r="O16" s="8" t="n"/>
+      <c r="P16" s="8" t="n"/>
+      <c r="Q16" s="8" t="n"/>
+      <c r="R16" s="8" t="n"/>
+      <c r="S16" s="8" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>Indeed</t>
+        </is>
+      </c>
+      <c r="B17" s="7" t="inlineStr">
+        <is>
+          <t>optometrist</t>
+        </is>
+      </c>
+      <c r="C17" s="7" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="n"/>
+      <c r="E17" s="8" t="n"/>
+      <c r="F17" s="8" t="n"/>
+      <c r="G17" s="8" t="n"/>
+      <c r="H17" s="8" t="n"/>
+      <c r="I17" s="8" t="n"/>
+      <c r="J17" s="8" t="n"/>
+      <c r="K17" s="8" t="n"/>
+      <c r="L17" s="8" t="n"/>
+      <c r="M17" s="8" t="n"/>
+      <c r="N17" s="8" t="n"/>
+      <c r="O17" s="8" t="n"/>
+      <c r="P17" s="8" t="n"/>
+      <c r="Q17" s="8" t="n"/>
+      <c r="R17" s="8" t="n"/>
+      <c r="S17" s="8" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="7" t="inlineStr">
+        <is>
+          <t>Indeed</t>
+        </is>
+      </c>
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>optician</t>
+        </is>
+      </c>
+      <c r="C18" s="7" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="D18" s="8" t="n"/>
+      <c r="E18" s="8" t="n"/>
+      <c r="F18" s="8" t="n"/>
+      <c r="G18" s="8" t="n"/>
+      <c r="H18" s="8" t="n"/>
+      <c r="I18" s="8" t="n"/>
+      <c r="J18" s="8" t="n"/>
+      <c r="K18" s="8" t="n"/>
+      <c r="L18" s="8" t="n"/>
+      <c r="M18" s="8" t="n"/>
+      <c r="N18" s="8" t="n"/>
+      <c r="O18" s="8" t="n"/>
+      <c r="P18" s="8" t="n"/>
+      <c r="Q18" s="8" t="n"/>
+      <c r="R18" s="8" t="n"/>
+      <c r="S18" s="8" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="7" t="inlineStr">
+        <is>
+          <t>Indeed</t>
+        </is>
+      </c>
+      <c r="B19" s="7" t="inlineStr">
+        <is>
+          <t>optometric assistant</t>
+        </is>
+      </c>
+      <c r="C19" s="7" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="D19" s="8" t="n"/>
+      <c r="E19" s="8" t="n"/>
+      <c r="F19" s="8" t="n"/>
+      <c r="G19" s="8" t="n"/>
+      <c r="H19" s="8" t="n"/>
+      <c r="I19" s="8" t="n"/>
+      <c r="J19" s="8" t="n"/>
+      <c r="K19" s="8" t="n"/>
+      <c r="L19" s="8" t="n"/>
+      <c r="M19" s="8" t="n"/>
+      <c r="N19" s="8" t="n"/>
+      <c r="O19" s="8" t="n"/>
+      <c r="P19" s="8" t="n"/>
+      <c r="Q19" s="8" t="n"/>
+      <c r="R19" s="8" t="n"/>
+      <c r="S19" s="8" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="7" t="inlineStr">
+        <is>
+          <t>Indeed</t>
+        </is>
+      </c>
+      <c r="B20" s="7" t="inlineStr">
+        <is>
+          <t>optometric technician</t>
+        </is>
+      </c>
+      <c r="C20" s="7" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="D20" s="8" t="n"/>
+      <c r="E20" s="8" t="n"/>
+      <c r="F20" s="8" t="n"/>
+      <c r="G20" s="8" t="n"/>
+      <c r="H20" s="8" t="n"/>
+      <c r="I20" s="8" t="n"/>
+      <c r="J20" s="8" t="n"/>
+      <c r="K20" s="8" t="n"/>
+      <c r="L20" s="8" t="n"/>
+      <c r="M20" s="8" t="n"/>
+      <c r="N20" s="8" t="n"/>
+      <c r="O20" s="8" t="n"/>
+      <c r="P20" s="8" t="n"/>
+      <c r="Q20" s="8" t="n"/>
+      <c r="R20" s="8" t="n"/>
+      <c r="S20" s="8" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="7" t="inlineStr">
+        <is>
+          <t>Indeed</t>
+        </is>
+      </c>
+      <c r="B21" s="7" t="inlineStr">
+        <is>
+          <t>ophthalmic assistant</t>
+        </is>
+      </c>
+      <c r="C21" s="7" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="D21" s="8" t="n"/>
+      <c r="E21" s="8" t="n"/>
+      <c r="F21" s="8" t="n"/>
+      <c r="G21" s="8" t="n"/>
+      <c r="H21" s="8" t="n"/>
+      <c r="I21" s="8" t="n"/>
+      <c r="J21" s="8" t="n"/>
+      <c r="K21" s="8" t="n"/>
+      <c r="L21" s="8" t="n"/>
+      <c r="M21" s="8" t="n"/>
+      <c r="N21" s="8" t="n"/>
+      <c r="O21" s="8" t="n"/>
+      <c r="P21" s="8" t="n"/>
+      <c r="Q21" s="8" t="n"/>
+      <c r="R21" s="8" t="n"/>
+      <c r="S21" s="8" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="7" t="inlineStr">
+        <is>
+          <t>Indeed</t>
+        </is>
+      </c>
+      <c r="B22" s="7" t="inlineStr">
+        <is>
+          <t>optical manager</t>
+        </is>
+      </c>
+      <c r="C22" s="7" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="D22" s="8" t="n"/>
+      <c r="E22" s="8" t="n"/>
+      <c r="F22" s="8" t="n"/>
+      <c r="G22" s="8" t="n"/>
+      <c r="H22" s="8" t="n"/>
+      <c r="I22" s="8" t="n"/>
+      <c r="J22" s="8" t="n"/>
+      <c r="K22" s="8" t="n"/>
+      <c r="L22" s="8" t="n"/>
+      <c r="M22" s="8" t="n"/>
+      <c r="N22" s="8" t="n"/>
+      <c r="O22" s="8" t="n"/>
+      <c r="P22" s="8" t="n"/>
+      <c r="Q22" s="8" t="n"/>
+      <c r="R22" s="8" t="n"/>
+      <c r="S22" s="8" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="7" t="inlineStr">
+        <is>
+          <t>Indeed</t>
+        </is>
+      </c>
+      <c r="B23" s="7" t="inlineStr">
+        <is>
+          <t>eye care clinic</t>
+        </is>
+      </c>
+      <c r="C23" s="7" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="D23" s="8" t="n"/>
+      <c r="E23" s="8" t="n"/>
+      <c r="F23" s="8" t="n"/>
+      <c r="G23" s="8" t="n"/>
+      <c r="H23" s="8" t="n"/>
+      <c r="I23" s="8" t="n"/>
+      <c r="J23" s="8" t="n"/>
+      <c r="K23" s="8" t="n"/>
+      <c r="L23" s="8" t="n"/>
+      <c r="M23" s="8" t="n"/>
+      <c r="N23" s="8" t="n"/>
+      <c r="O23" s="8" t="n"/>
+      <c r="P23" s="8" t="n"/>
+      <c r="Q23" s="8" t="n"/>
+      <c r="R23" s="8" t="n"/>
+      <c r="S23" s="8" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="7" t="inlineStr">
+        <is>
+          <t>(your own)</t>
+        </is>
+      </c>
+      <c r="B24" s="9" t="inlineStr"/>
+      <c r="C24" s="7" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="D24" s="8" t="n"/>
+      <c r="E24" s="8" t="n"/>
+      <c r="F24" s="8" t="n"/>
+      <c r="G24" s="8" t="n"/>
+      <c r="H24" s="8" t="n"/>
+      <c r="I24" s="8" t="n"/>
+      <c r="J24" s="8" t="n"/>
+      <c r="K24" s="8" t="n"/>
+      <c r="L24" s="8" t="n"/>
+      <c r="M24" s="8" t="n"/>
+      <c r="N24" s="8" t="n"/>
+      <c r="O24" s="8" t="n"/>
+      <c r="P24" s="8" t="n"/>
+      <c r="Q24" s="8" t="n"/>
+      <c r="R24" s="8" t="n"/>
+      <c r="S24" s="8" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="10" t="inlineStr">
         <is>
           <t>Total, all rows</t>
         </is>
       </c>
-      <c r="D16" s="11">
-        <f>IF(COUNT(D5:D14)=0,"",SUM(D5:D14))</f>
-        <v/>
-      </c>
-      <c r="E16" s="11">
-        <f>IF(COUNT(E5:E14)=0,"",SUM(E5:E14))</f>
-        <v/>
-      </c>
-      <c r="F16" s="11">
-        <f>IF(COUNT(F5:F14)=0,"",SUM(F5:F14))</f>
-        <v/>
-      </c>
-      <c r="G16" s="11">
-        <f>IF(COUNT(G5:G14)=0,"",SUM(G5:G14))</f>
-        <v/>
-      </c>
-      <c r="H16" s="11">
-        <f>IF(COUNT(H5:H14)=0,"",SUM(H5:H14))</f>
-        <v/>
-      </c>
-      <c r="I16" s="11">
-        <f>IF(COUNT(I5:I14)=0,"",SUM(I5:I14))</f>
-        <v/>
-      </c>
-      <c r="J16" s="11">
-        <f>IF(COUNT(J5:J14)=0,"",SUM(J5:J14))</f>
-        <v/>
-      </c>
-      <c r="K16" s="11">
-        <f>IF(COUNT(K5:K14)=0,"",SUM(K5:K14))</f>
-        <v/>
-      </c>
-      <c r="L16" s="11">
-        <f>IF(COUNT(L5:L14)=0,"",SUM(L5:L14))</f>
-        <v/>
-      </c>
-      <c r="M16" s="11">
-        <f>IF(COUNT(M5:M14)=0,"",SUM(M5:M14))</f>
-        <v/>
-      </c>
-      <c r="N16" s="11">
-        <f>IF(COUNT(N5:N14)=0,"",SUM(N5:N14))</f>
-        <v/>
-      </c>
-      <c r="O16" s="11">
-        <f>IF(COUNT(O5:O14)=0,"",SUM(O5:O14))</f>
-        <v/>
-      </c>
-      <c r="P16" s="11">
-        <f>IF(COUNT(P5:P14)=0,"",SUM(P5:P14))</f>
-        <v/>
-      </c>
-      <c r="Q16" s="11">
-        <f>IF(COUNT(Q5:Q14)=0,"",SUM(Q5:Q14))</f>
-        <v/>
-      </c>
-      <c r="R16" s="11">
-        <f>IF(COUNT(R5:R14)=0,"",SUM(R5:R14))</f>
-        <v/>
-      </c>
-      <c r="S16" s="11">
-        <f>IF(COUNT(S5:S14)=0,"",SUM(S5:S14))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="10" t="inlineStr">
+      <c r="D26" s="11">
+        <f>IF(COUNT(D5:D24)=0,"",SUM(D5:D24))</f>
+        <v/>
+      </c>
+      <c r="E26" s="11">
+        <f>IF(COUNT(E5:E24)=0,"",SUM(E5:E24))</f>
+        <v/>
+      </c>
+      <c r="F26" s="11">
+        <f>IF(COUNT(F5:F24)=0,"",SUM(F5:F24))</f>
+        <v/>
+      </c>
+      <c r="G26" s="11">
+        <f>IF(COUNT(G5:G24)=0,"",SUM(G5:G24))</f>
+        <v/>
+      </c>
+      <c r="H26" s="11">
+        <f>IF(COUNT(H5:H24)=0,"",SUM(H5:H24))</f>
+        <v/>
+      </c>
+      <c r="I26" s="11">
+        <f>IF(COUNT(I5:I24)=0,"",SUM(I5:I24))</f>
+        <v/>
+      </c>
+      <c r="J26" s="11">
+        <f>IF(COUNT(J5:J24)=0,"",SUM(J5:J24))</f>
+        <v/>
+      </c>
+      <c r="K26" s="11">
+        <f>IF(COUNT(K5:K24)=0,"",SUM(K5:K24))</f>
+        <v/>
+      </c>
+      <c r="L26" s="11">
+        <f>IF(COUNT(L5:L24)=0,"",SUM(L5:L24))</f>
+        <v/>
+      </c>
+      <c r="M26" s="11">
+        <f>IF(COUNT(M5:M24)=0,"",SUM(M5:M24))</f>
+        <v/>
+      </c>
+      <c r="N26" s="11">
+        <f>IF(COUNT(N5:N24)=0,"",SUM(N5:N24))</f>
+        <v/>
+      </c>
+      <c r="O26" s="11">
+        <f>IF(COUNT(O5:O24)=0,"",SUM(O5:O24))</f>
+        <v/>
+      </c>
+      <c r="P26" s="11">
+        <f>IF(COUNT(P5:P24)=0,"",SUM(P5:P24))</f>
+        <v/>
+      </c>
+      <c r="Q26" s="11">
+        <f>IF(COUNT(Q5:Q24)=0,"",SUM(Q5:Q24))</f>
+        <v/>
+      </c>
+      <c r="R26" s="11">
+        <f>IF(COUNT(R5:R24)=0,"",SUM(R5:R24))</f>
+        <v/>
+      </c>
+      <c r="S26" s="11">
+        <f>IF(COUNT(S5:S24)=0,"",SUM(S5:S24))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="10" t="inlineStr">
         <is>
           <t>Notes for each week (anything odd: a holiday, a site change, a search that behaved differently):</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="12" t="n"/>
-    </row>
-    <row r="20"/>
-    <row r="21"/>
+    <row r="29">
+      <c r="A29" s="12" t="n"/>
+    </row>
+    <row r="30"/>
+    <row r="31"/>
   </sheetData>
   <mergeCells count="9">
     <mergeCell ref="F3:G3"/>
@@ -1202,9 +1532,9 @@
     <mergeCell ref="J3:K3"/>
     <mergeCell ref="P3:Q3"/>
     <mergeCell ref="N3:O3"/>
-    <mergeCell ref="A19:S21"/>
     <mergeCell ref="R3:S3"/>
     <mergeCell ref="D3:E3"/>
+    <mergeCell ref="A29:S31"/>
     <mergeCell ref="H3:I3"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1245,7 +1575,7 @@
         </is>
       </c>
       <c r="B4">
-        <f>COUNT(Counts!D16,Counts!F16,Counts!H16,Counts!J16,Counts!L16,Counts!N16,Counts!P16,Counts!R16)</f>
+        <f>COUNT(Counts!D26,Counts!F26,Counts!H26,Counts!J26,Counts!L26,Counts!N26,Counts!P26,Counts!R26)</f>
         <v/>
       </c>
     </row>
@@ -1256,7 +1586,7 @@
         </is>
       </c>
       <c r="B5">
-        <f>IF(B4=0,"",AVERAGE(Counts!D16,Counts!F16,Counts!H16,Counts!J16,Counts!L16,Counts!N16,Counts!P16,Counts!R16))</f>
+        <f>IF(B4=0,"",AVERAGE(Counts!D26,Counts!F26,Counts!H26,Counts!J26,Counts!L26,Counts!N26,Counts!P26,Counts!R26))</f>
         <v/>
       </c>
     </row>
@@ -1267,7 +1597,7 @@
         </is>
       </c>
       <c r="B6">
-        <f>IF(COUNT(Counts!E16,Counts!G16,Counts!I16,Counts!K16,Counts!M16,Counts!O16,Counts!Q16,Counts!S16)=0,"",AVERAGE(Counts!E16,Counts!G16,Counts!I16,Counts!K16,Counts!M16,Counts!O16,Counts!Q16,Counts!S16))</f>
+        <f>IF(COUNT(Counts!E26,Counts!G26,Counts!I26,Counts!K26,Counts!M26,Counts!O26,Counts!Q26,Counts!S26)=0,"",AVERAGE(Counts!E26,Counts!G26,Counts!I26,Counts!K26,Counts!M26,Counts!O26,Counts!Q26,Counts!S26))</f>
         <v/>
       </c>
     </row>

</xml_diff>